<commit_message>
add dockerfile for deployment
</commit_message>
<xml_diff>
--- a/documentation/Jira_Backlog_English_to_Hindi_Translator.xlsx
+++ b/documentation/Jira_Backlog_English_to_Hindi_Translator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\college\GitHubINV\aitranslator_webapp\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFF050E6-7CB7-4D25-8DF6-8545FAE1811C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E191004-F2DB-4BF0-AE70-92AFD82E0CF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -637,7 +637,7 @@
         <v>14</v>
       </c>
       <c r="I3" t="s">
-        <v>15</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>